<commit_message>
update docs styling (again) ! fix release fixtures version update process
</commit_message>
<xml_diff>
--- a/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product_multi_source_sample.xlsx
+++ b/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product_multi_source_sample.xlsx
@@ -1,36 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fundamentals" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schema stg_customers" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SLA" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Servers" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pricing" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Custom Properties" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Models" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Model Inputs" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Sources" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Source Schema" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Mapping" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Parameters" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Relationships" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operational Validation" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operational Parameters" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Lookups" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Build" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_DET Lists" sheetId="24" state="veryHidden" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_DET Metadata" sheetId="25" state="veryHidden" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_DET Context" sheetId="26" state="veryHidden" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_DET Raw ODCS" sheetId="27" state="veryHidden" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schema customer_account_mart" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Fundamentals" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Schema stg_customers" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Relationships" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Quality" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Support" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Team" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Roles" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="SLA" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Servers" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Pricing" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Custom Properties" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="DET Models" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="DET Model Inputs" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="DET Sources" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="DET Source Schema" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="DET Mapping" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="DET Parameters" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="DET Relationships" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Operational Validation" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Operational Parameters" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="DET Lookups" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="DET Build" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="_DET Lists" sheetId="24" state="veryHidden" r:id="rId24"/>
+    <sheet name="_DET Metadata" sheetId="25" state="veryHidden" r:id="rId25"/>
+    <sheet name="_DET Context" sheetId="26" state="veryHidden" r:id="rId26"/>
+    <sheet name="_DET Raw ODCS" sheetId="27" state="veryHidden" r:id="rId27"/>
+    <sheet name="Schema customer_account_mart" sheetId="28" state="visible" r:id="rId28"/>
   </sheets>
   <definedNames>
     <definedName name="apiVersion">Fundamentals!$C$5</definedName>
@@ -15587,7 +15587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="189" min="1" max="1"/>
@@ -15628,7 +15628,7 @@
       </c>
       <c r="B4" s="193" t="inlineStr">
         <is>
-          <t>2.3.0</t>
+          <t>3.0.2</t>
         </is>
       </c>
     </row>
@@ -15640,7 +15640,7 @@
       </c>
       <c r="B5" s="193" t="inlineStr">
         <is>
-          <t>2.3.0</t>
+          <t>3.0.2</t>
         </is>
       </c>
     </row>
@@ -15652,7 +15652,7 @@
       </c>
       <c r="B6" s="193" t="inlineStr">
         <is>
-          <t>2.3.0</t>
+          <t>3.0.2</t>
         </is>
       </c>
     </row>
@@ -15664,7 +15664,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>1429ce4f80e5f9adf552a3fd404d94b7e7a0cd98434fff6fafe63717a8a6b8cf</t>
+          <t>63d2b950ce8bbc71970b53ea88f565f4b1316accc4ff288ace05532edfc75182</t>
         </is>
       </c>
     </row>
@@ -15680,6 +15680,10 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CCB4"/>
   <mergeCells count="2">
@@ -15932,11 +15936,15 @@
           <t>_det_invocation_id</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>Remove Prefix</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
           <t>Precision</t>
@@ -15952,6 +15960,8 @@
           <t>Trim</t>
         </is>
       </c>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
           <t>Lookup</t>
@@ -15982,21 +15992,29 @@
           <t>Allow Null</t>
         </is>
       </c>
+      <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr">
         <is>
           <t>Lookup</t>
         </is>
       </c>
+      <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr">
         <is>
           <t>Pattern</t>
         </is>
       </c>
+      <c r="Z2" t="inlineStr"/>
       <c r="AA2" t="inlineStr">
         <is>
           <t>Operator</t>
         </is>
       </c>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
       <c r="AG2" t="inlineStr">
         <is>
           <t>_det_invocation_id</t>
@@ -20776,7 +20794,16 @@
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="B10:E10"/>
   </mergeCells>
-  <dataValidations count="9">
+  <dataValidations count="12">
+    <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
+      <formula1>'_DET Lists'!$U$2:$U$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
+      <formula1>'_DET Lists'!$U$2:$U$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
+      <formula1>'_DET Lists'!$U$2:$U$4</formula1>
+    </dataValidation>
     <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
       <formula1>'_DET Lists'!$U$2:$U$4</formula1>
     </dataValidation>
@@ -25019,7 +25046,16 @@
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="B10:E10"/>
   </mergeCells>
-  <dataValidations count="20">
+  <dataValidations count="23">
+    <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
+      <formula1>'_DET Lists'!$U$2:$U$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
+      <formula1>'_DET Lists'!$U$2:$U$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
+      <formula1>'_DET Lists'!$U$2:$U$4</formula1>
+    </dataValidation>
     <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
       <formula1>'_DET Lists'!$U$2:$U$4</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
update release fixture generation! and updated flow
</commit_message>
<xml_diff>
--- a/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product_multi_source_sample.xlsx
+++ b/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product_multi_source_sample.xlsx
@@ -15628,7 +15628,7 @@
       </c>
       <c r="B4" s="193" t="inlineStr">
         <is>
-          <t>3.0.2</t>
+          <t>3.0.3</t>
         </is>
       </c>
     </row>
@@ -15640,7 +15640,7 @@
       </c>
       <c r="B5" s="193" t="inlineStr">
         <is>
-          <t>3.0.2</t>
+          <t>3.0.3</t>
         </is>
       </c>
     </row>
@@ -15652,7 +15652,7 @@
       </c>
       <c r="B6" s="193" t="inlineStr">
         <is>
-          <t>3.0.2</t>
+          <t>3.0.3</t>
         </is>
       </c>
     </row>
@@ -15664,7 +15664,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>63d2b950ce8bbc71970b53ea88f565f4b1316accc4ff288ace05532edfc75182</t>
+          <t>bf4c150acbff83880b41db78850d5e09436aa99c889805695f1d7a8a2b90bbeb</t>
         </is>
       </c>
     </row>
@@ -20794,7 +20794,10 @@
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="B10:E10"/>
   </mergeCells>
-  <dataValidations count="12">
+  <dataValidations count="13">
+    <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
+      <formula1>'_DET Lists'!$U$2:$U$4</formula1>
+    </dataValidation>
     <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
       <formula1>'_DET Lists'!$U$2:$U$4</formula1>
     </dataValidation>
@@ -25046,7 +25049,10 @@
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="B10:E10"/>
   </mergeCells>
-  <dataValidations count="23">
+  <dataValidations count="24">
+    <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
+      <formula1>'_DET Lists'!$U$2:$U$4</formula1>
+    </dataValidation>
     <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
       <formula1>'_DET Lists'!$U$2:$U$4</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
fixed release flow issue for bumpver! because files were not committed!
</commit_message>
<xml_diff>
--- a/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product_multi_source_sample.xlsx
+++ b/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product_multi_source_sample.xlsx
@@ -15628,7 +15628,7 @@
       </c>
       <c r="B4" s="193" t="inlineStr">
         <is>
-          <t>3.0.3</t>
+          <t>3.0.4</t>
         </is>
       </c>
     </row>
@@ -15640,7 +15640,7 @@
       </c>
       <c r="B5" s="193" t="inlineStr">
         <is>
-          <t>3.0.3</t>
+          <t>3.0.4</t>
         </is>
       </c>
     </row>
@@ -15652,7 +15652,7 @@
       </c>
       <c r="B6" s="193" t="inlineStr">
         <is>
-          <t>3.0.3</t>
+          <t>3.0.4</t>
         </is>
       </c>
     </row>
@@ -15664,7 +15664,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>bf4c150acbff83880b41db78850d5e09436aa99c889805695f1d7a8a2b90bbeb</t>
+          <t>ac3ea59527188645c7771fc723c3cb1676c83b06370a8318092dc82bdee5ddcd</t>
         </is>
       </c>
     </row>
@@ -20794,7 +20794,13 @@
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="B10:E10"/>
   </mergeCells>
-  <dataValidations count="13">
+  <dataValidations count="15">
+    <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
+      <formula1>'_DET Lists'!$U$2:$U$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
+      <formula1>'_DET Lists'!$U$2:$U$4</formula1>
+    </dataValidation>
     <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
       <formula1>'_DET Lists'!$U$2:$U$4</formula1>
     </dataValidation>
@@ -25049,7 +25055,13 @@
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="B10:E10"/>
   </mergeCells>
-  <dataValidations count="24">
+  <dataValidations count="26">
+    <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
+      <formula1>'_DET Lists'!$U$2:$U$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
+      <formula1>'_DET Lists'!$U$2:$U$4</formula1>
+    </dataValidation>
     <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
       <formula1>'_DET Lists'!$U$2:$U$4</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
bump version 3.0.4 -> 3.0.5
</commit_message>
<xml_diff>
--- a/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product_multi_source_sample.xlsx
+++ b/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product_multi_source_sample.xlsx
@@ -15628,7 +15628,7 @@
       </c>
       <c r="B4" s="193" t="inlineStr">
         <is>
-          <t>3.0.4</t>
+          <t>3.0.5</t>
         </is>
       </c>
     </row>
@@ -15640,7 +15640,7 @@
       </c>
       <c r="B5" s="193" t="inlineStr">
         <is>
-          <t>3.0.4</t>
+          <t>3.0.5</t>
         </is>
       </c>
     </row>
@@ -15652,7 +15652,7 @@
       </c>
       <c r="B6" s="193" t="inlineStr">
         <is>
-          <t>3.0.4</t>
+          <t>3.0.5</t>
         </is>
       </c>
     </row>
@@ -15664,7 +15664,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ac3ea59527188645c7771fc723c3cb1676c83b06370a8318092dc82bdee5ddcd</t>
+          <t>80864bd3c138d9b186867baa0b5789dbe2f5aecacac3e1882fb0214611f059c6</t>
         </is>
       </c>
     </row>
@@ -20794,7 +20794,10 @@
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="B10:E10"/>
   </mergeCells>
-  <dataValidations count="15">
+  <dataValidations count="16">
+    <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
+      <formula1>'_DET Lists'!$U$2:$U$4</formula1>
+    </dataValidation>
     <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
       <formula1>'_DET Lists'!$U$2:$U$4</formula1>
     </dataValidation>
@@ -25055,7 +25058,10 @@
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="B10:E10"/>
   </mergeCells>
-  <dataValidations count="26">
+  <dataValidations count="27">
+    <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
+      <formula1>'_DET Lists'!$U$2:$U$4</formula1>
+    </dataValidation>
     <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
       <formula1>'_DET Lists'!$U$2:$U$4</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
update the release fixtures to include changelog
</commit_message>
<xml_diff>
--- a/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product_multi_source_sample.xlsx
+++ b/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product_multi_source_sample.xlsx
@@ -14537,7 +14537,7 @@
       </c>
       <c r="B8" s="207" t="inlineStr">
         <is>
-          <t>v2.3.0</t>
+          <t>v3.0.5</t>
         </is>
       </c>
       <c r="C8" s="193" t="inlineStr">
@@ -20794,7 +20794,10 @@
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="B10:E10"/>
   </mergeCells>
-  <dataValidations count="16">
+  <dataValidations count="17">
+    <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
+      <formula1>'_DET Lists'!$U$2:$U$4</formula1>
+    </dataValidation>
     <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
       <formula1>'_DET Lists'!$U$2:$U$4</formula1>
     </dataValidation>
@@ -25058,7 +25061,10 @@
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="B10:E10"/>
   </mergeCells>
-  <dataValidations count="27">
+  <dataValidations count="28">
+    <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
+      <formula1>'_DET Lists'!$U$2:$U$4</formula1>
+    </dataValidation>
     <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
       <formula1>'_DET Lists'!$U$2:$U$4</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
bump version 3.0.5 -> 3.0.6
</commit_message>
<xml_diff>
--- a/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product_multi_source_sample.xlsx
+++ b/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product_multi_source_sample.xlsx
@@ -14537,7 +14537,7 @@
       </c>
       <c r="B8" s="207" t="inlineStr">
         <is>
-          <t>v3.0.5</t>
+          <t>v3.0.6</t>
         </is>
       </c>
       <c r="C8" s="193" t="inlineStr">
@@ -15628,7 +15628,7 @@
       </c>
       <c r="B4" s="193" t="inlineStr">
         <is>
-          <t>3.0.5</t>
+          <t>3.0.6</t>
         </is>
       </c>
     </row>
@@ -15640,7 +15640,7 @@
       </c>
       <c r="B5" s="193" t="inlineStr">
         <is>
-          <t>3.0.5</t>
+          <t>3.0.6</t>
         </is>
       </c>
     </row>
@@ -15652,7 +15652,7 @@
       </c>
       <c r="B6" s="193" t="inlineStr">
         <is>
-          <t>3.0.5</t>
+          <t>3.0.6</t>
         </is>
       </c>
     </row>
@@ -15664,7 +15664,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>80864bd3c138d9b186867baa0b5789dbe2f5aecacac3e1882fb0214611f059c6</t>
+          <t>3385d149ed874f52ab9eaebff1fcea94dbdf2bf04554c8714bbee079d7b75cc1</t>
         </is>
       </c>
     </row>
@@ -20794,7 +20794,10 @@
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="B10:E10"/>
   </mergeCells>
-  <dataValidations count="17">
+  <dataValidations count="18">
+    <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
+      <formula1>'_DET Lists'!$U$2:$U$4</formula1>
+    </dataValidation>
     <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
       <formula1>'_DET Lists'!$U$2:$U$4</formula1>
     </dataValidation>
@@ -25061,7 +25064,10 @@
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="B10:E10"/>
   </mergeCells>
-  <dataValidations count="28">
+  <dataValidations count="29">
+    <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
+      <formula1>'_DET Lists'!$U$2:$U$4</formula1>
+    </dataValidation>
     <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
       <formula1>'_DET Lists'!$U$2:$U$4</formula1>
     </dataValidation>

</xml_diff>